<commit_message>
Refine first-floor enemy roster and monster table
</commit_message>
<xml_diff>
--- a/怪物配置表.xlsx
+++ b/怪物配置表.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'怪物配置总表'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'第一层配置'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'第一层数值基准'!$A$1:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段说明'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'怪物配置总表'!$A$1:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'第一层配置'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'第一层数值基准'!$A$1:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段说明'!$A$1:$B$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,8 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,6 +514,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>素材路径</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>状态</t>
         </is>
       </c>
@@ -525,7 +531,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -539,11 +545,11 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>攻击[7] / 防御[7]</t>
+          <t>攻击[6] / 防御[5]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -553,24 +559,29 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>第一场教学怪，验证攻击、防御、多行敌方编码区和意图预览</t>
+          <t>第一层基础攻防教学，验证敌方代码、多行意图和护盾窗口</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>已实装</t>
+          <t>img/enemies/bug.png</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>数值已实装；新素材待接入</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>typo</t>
+          <t>error</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>错字虫</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -588,34 +599,39 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>攻击[6-9]</t>
+          <t>攻击[7-10]</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>每回合小幅随机伤害</t>
+          <t>每回合只攻击；每次受到攻击有 10% 概率下回合眩晕</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>引入随机伤害，但压力较低</t>
+          <t>高一点的随机攻击压力，鼓励玩家主动攻击并理解打断机会</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>已实装</t>
+          <t>img/enemies/error.png</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>素材已生成；机制待接入</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>redpoint</t>
+          <t>loop</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>红点提醒</t>
+          <t>回环</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -629,38 +645,43 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>攻击[6] / 提醒弹出()</t>
+          <t>循环(2){攻击[3]} / 防御[5] / 循环(3){攻击[2]}</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>每 3 回合触发一次：下回合少抽 1 张牌</t>
+          <t>通过低伤害多段行动引入循环机制</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>轻度手牌干扰，让玩家感知下回合资源</t>
+          <t>让玩家第一次理解循环不是抽象语法，而是重复执行的敌方行动</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>已实装</t>
+          <t>img/enemies/loop.png</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>素材已生成；机制待接入</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>nullptr</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>空值幽影</t>
+          <t>岔路</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -670,42 +691,47 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>普通/精英</t>
+          <t>普通</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>攻击[8] / // 空值潜伏 / 攻击[12]</t>
+          <t>如果(你无护盾) 攻击[9] / 否则 攻击[5]</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>潜伏一回合后打出较高伤害</t>
+          <t>根据玩家状态改变行动，引入判断机制</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>教玩家看节奏，准备防御或爆发</t>
+          <t>教玩家用防御影响敌方分支，建立 if/else 的战斗直觉</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>已实装</t>
+          <t>img/enemies/branch.png</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>素材已生成；机制待接入</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>chaser</t>
+          <t>nullptr</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>催单员</t>
+          <t>空值</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -715,42 +741,43 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>普通/精英</t>
+          <t>精英候选</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>攻击[5+t*2]</t>
+          <t>攻击[7] / // 空值潜伏 / 攻击[11]</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>伤害随回合递增</t>
+          <t>潜伏一回合后打出较高伤害</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>拖延惩罚，逼玩家尽快结束战斗</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>已实装</t>
+          <t>后段或精英节点的节奏预判测试，暂不放入前段普通池</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>旧配置保留；待重命名/重做素材</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>chaser</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>待办残片</t>
+          <t>催单</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -760,87 +787,89 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>普通/精英</t>
+          <t>精英候选</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>攻击[9] / 防御[8]</t>
+          <t>攻击[4+t*2]</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>攻击与防御交替</t>
+          <t>伤害随回合递增</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>教玩家识别敌方防御回合和输出窗口</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>已实装</t>
+          <t>拖延惩罚，逼玩家尽快结束战斗</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>旧配置保留；待重做素材</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>infloop</t>
+          <t>todo</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>InfiniteLoop</t>
+          <t>待办</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>第二层</t>
+          <t>第一层</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>普通</t>
+          <t>精英候选</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>攻击[3+t*2]</t>
+          <t>攻击[8] / 防御[7]</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>伤害随回合线性成长</t>
+          <t>攻击与防御交替</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>第二层成长压力怪</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>待重命名</t>
+          <t>教玩家识别敌方防御回合和输出窗口</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>旧配置保留；待重做素材</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>memleak</t>
+          <t>infloop</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>MemoryLeak</t>
+          <t>InfiniteLoop</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -854,24 +883,25 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>吸血[4-6]</t>
+          <t>攻击[3+t*2]</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>造成伤害后回复一半生命</t>
+          <t>伤害随回合线性成长</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>拖延惩罚，要求稳定输出</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+          <t>第二层成长压力怪</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -880,43 +910,44 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>recursion</t>
+          <t>memleak</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>MemoryLeak</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>第二/三层</t>
+          <t>第二层</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>精英</t>
+          <t>普通</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>攻击[5,10,20,40]</t>
+          <t>吸血[4-6]</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>伤害指数增长，上限 40</t>
+          <t>造成伤害后回复一半生命</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>强爆发预警怪</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
+          <t>拖延惩罚，要求稳定输出</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -925,12 +956,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>stackoverflow</t>
+          <t>recursion</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>StackOverflow</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -944,24 +975,25 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>循环(3){攻击[4]}</t>
+          <t>攻击[5,10,20,40]</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>多段攻击，总伤害 12</t>
+          <t>伤害指数增长，上限 40</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>检验护盾、反弹和多段防御能力</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+          <t>强爆发预警怪</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -970,12 +1002,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>racecond</t>
+          <t>stackoverflow</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>RaceCondition</t>
+          <t>StackOverflow</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -985,28 +1017,29 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>普通</t>
+          <t>精英</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>攻击[3-20] // 随机</t>
+          <t>循环(3){攻击[4]}</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>伤害大幅随机，但会提前显示本回合数值</t>
+          <t>多段攻击，总伤害 12</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>高波动风险怪</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+          <t>检验护盾、反弹和多段防御能力</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -1015,12 +1048,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>deadlock</t>
+          <t>racecond</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Deadlock</t>
+          <t>RaceCondition</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1030,28 +1063,29 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>精英</t>
+          <t>普通</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>防御[15] / 攻击[20]</t>
+          <t>攻击[3-20] // 随机</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>防御与重击交替</t>
+          <t>伤害大幅随机，但会提前显示本回合数值</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>窗口型战斗，鼓励破盾和爆发</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+          <t>高波动风险怪</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -1060,12 +1094,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>gc</t>
+          <t>deadlock</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GarbageCollector</t>
+          <t>Deadlock</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1075,28 +1109,29 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>普通</t>
+          <t>精英</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>垃圾回收() / 攻击[6-10]</t>
+          <t>防御[15] / 攻击[20]</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>偶数回合移除 1 张手牌</t>
+          <t>防御与重击交替</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>手牌资源干扰</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
+          <t>窗口型战斗，鼓励破盾和爆发</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
@@ -1105,62 +1140,63 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>syntaxerr</t>
+          <t>gc</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>红字审判</t>
+          <t>GarbageCollector</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>第一层</t>
+          <t>第二/三层</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>普通</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>140</v>
+        <v>35</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>防御[12] / 攻击[12-18] / 语法错误!</t>
+          <t>垃圾回收() / 攻击[6-10]</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>周期性护盾、攻击、随机弃 1 张手牌</t>
+          <t>偶数回合移除 1 张手牌</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>第一层综合检验 Boss</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>已实装</t>
+          <t>手牌资源干扰</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>待重命名</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>firewall</t>
+          <t>syntaxerr</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Firewall</t>
+          <t>红字</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>第二层</t>
+          <t>第一层</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1169,76 +1205,124 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>防御[20] / 防御[15]+攻击[10] / 攻击[25]</t>
+          <t>防御[10] / 攻击[10-15] / 语法错误!</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>高护盾与高爆发交替</t>
+          <t>周期性护盾、攻击、随机弃 1 张手牌</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>第二层护盾压力 Boss</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>待重命名</t>
+          <t>第一层综合检验 Boss</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>已实装；待重做素材</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Firewall</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>第二层</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>防御[20] / 防御[15]+攻击[10] / 攻击[25]</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>高护盾与高爆发交替</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>第二层护盾压力 Boss</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>待重命名</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>root</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Root</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>第三层</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Boss</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E18" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>循环(3){防御[10]} / 治疗[20] / 攻击[20-30]</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>护盾、治疗、高伤害循环</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>最终综合 Boss</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>待重命名</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1249,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1260,7 +1344,8 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1288,12 +1373,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>第一场教学</t>
+          <t>第一层前段普通池</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1303,41 +1388,41 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>HP 32；行动循环为攻击 7 -&gt; 防御 7 -&gt; 攻击 7 + 防御 7，适合教学敌方多行代码</t>
+          <t>HP 28；攻击/防御/攻击+防御循环，作为基础攻防教学</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>错字虫</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>第一层普通战</t>
+          <t>第一层前段普通池</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中低</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>HP 30，攻击 6-9；轻随机，不应造成强挫败</t>
+          <t>HP 30；攻击 7-10；受击 10% 概率下回合眩晕，压力稍高但有打断机会</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>红点提醒</t>
+          <t>回环</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>第一层中段</t>
+          <t>第一层第 3-4 列后加入</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1347,19 +1432,19 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>HP 34；少抽牌机制要让玩家感觉到，但不要频繁叠加</t>
+          <t>HP 32；低伤害多段行动，引入循环机制</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>空值幽影</t>
+          <t>岔路</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>第一层普通/精英</t>
+          <t>第一层第 3-4 列后加入</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1369,19 +1454,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>HP 38；潜伏后攻击，适合教预判</t>
+          <t>HP 34；根据玩家是否有护盾选择攻击强度，引入判断机制</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>催单员</t>
+          <t>空值</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>第一层精英或后段普通</t>
+          <t>第一层精英候选</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1391,19 +1476,19 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>HP 40；回合越久越危险</t>
+          <t>HP 38；潜伏后攻击，适合教预判；暂不进入前段普通池</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>待办残片</t>
+          <t>催单</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>第一层精英或后段普通</t>
+          <t>第一层精英候选</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1413,34 +1498,56 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>HP 42；防御回合给玩家观察窗口</t>
+          <t>HP 40；回合越久越危险</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>红字审判</t>
+          <t>待办</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>第一层精英候选</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>HP 40；防御回合给玩家观察窗口</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>红字</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>第一层 Boss</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>中高</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>HP 140；目标 6-8 回合战斗</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>HP 125；目标 6-8 回合战斗；后续需统一新美术风格</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1451,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1462,7 +1569,8 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1490,12 +1598,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>30-42</t>
+          <t>28-34</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>第一层普通战斗不要 1-2 回合结束</t>
+          <t>第一层普通战斗控制在约 3-4 回合，优先教学而非消耗</t>
         </is>
       </c>
     </row>
@@ -1507,119 +1615,136 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>6-9</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>玩家需要考虑防御，但不应被早期秒杀</t>
+          <t>玩家需要考虑防御，但不应被早期连续压血</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>普通怪强攻击</t>
+          <t>普通怪压力攻击</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>7-10</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>必须有预告或节奏提示</t>
+          <t>放在 Error 或带条件的岔路中，必须能通过主动攻击/防御缓解</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>第一层精英 HP</t>
+          <t>循环/判断引入</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>38-42 起步，后续可提高到 50-65</t>
+          <t>第 3-4 列后</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>当前先用普通怪精英化，后续可拆独立精英版本</t>
+          <t>先让玩家理解基础攻防，再引入 Loop 和 If 的敌方机制</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>第一层 Boss HP</t>
+          <t>第一层精英 HP</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>38-40</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>目标 6-8 回合</t>
+          <t>普通战不再抽精英怪，精英节点承担节奏测试</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>第一层 Boss 攻击</t>
+          <t>第一层 Boss HP</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>12-18</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>覆盖防御检查和血量压力</t>
+          <t>目标 6-8 回合</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>普通战斗目标时长</t>
+          <t>第一层 Boss 攻击</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3-4 回合</t>
+          <t>10-15</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>让机制有时间出现</t>
+          <t>覆盖防御检查和血量压力</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>普通战斗目标时长</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3-4 回合</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>让机制有时间出现</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Boss 战目标时长</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>6-8 回合</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>第一层综合检验</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C9"/>
+  <autoFilter ref="A1:C10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1630,7 +1755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1641,7 +1766,8 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1755,17 +1881,29 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>素材路径</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>透明 PNG 或后续美术资源路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>已实装、待重命名、待调整等</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update first-floor enemy configs and table
</commit_message>
<xml_diff>
--- a/怪物配置表.xlsx
+++ b/怪物配置表.xlsx
@@ -649,12 +649,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>循环(2){攻击[3]} / 防御[5] / 循环(3){攻击[2]}</t>
+          <t>①循环(3){攻击[3]} / ②循环(2){攻击[3] + 防御[3]}</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>通过低伤害多段行动引入循环机制</t>
+          <t>通过固定多段行动引入循环机制；第二段循环同时攻击与防御</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -699,12 +699,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>如果(你无护盾) 攻击[9] / 否则 攻击[5]</t>
+          <t>①攻击[3]；如果(你没有护盾) 攻击[5]；如果(自身HP&lt;30%) 攻击[3] / ②如果(你有护盾) 防御[5]；否则 下次攻击参数+1</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>根据玩家状态改变行动，引入判断机制</t>
+          <t>根据玩家护盾与自身血量走不同分支；无护盾时追击，低血量时补刀，有护盾时转防御，否则蓄积参数</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>HP 32；低伤害多段行动，引入循环机制</t>
+          <t>HP 32；①循环 3 次攻击 3；②循环 2 次攻击 3 + 防御 3，引入循环机制</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>HP 34；根据玩家是否有护盾选择攻击强度，引入判断机制</t>
+          <t>HP 34；①先攻击 3，再按玩家护盾/自身低血量判断追加攻击；②根据玩家是否有护盾选择防御或下次攻击参数+1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish first-floor demo and refresh enemy art
</commit_message>
<xml_diff>
--- a/怪物配置表.xlsx
+++ b/怪物配置表.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>数值已实装；新素材待接入</t>
+          <t>已接入</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>素材已生成；机制待接入</t>
+          <t>已接入</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>素材已生成；机制待接入</t>
+          <t>已接入</t>
         </is>
       </c>
     </row>
@@ -719,19 +719,19 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>素材已生成；机制待接入</t>
+          <t>已接入</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>nullptr</t>
+          <t>ddl</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>空值</t>
+          <t>DDL</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -741,31 +741,31 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>精英候选</t>
+          <t>精英</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>攻击[7] / // 空值潜伏 / 攻击[11]</t>
+          <t>攻击[6] / 易伤[1] / 攻击[12]</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>潜伏一回合后打出较高伤害</t>
+          <t>倒计时式精英；先施加 1 层易伤，再用大攻击制造截止压力</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>后段或精英节点的节奏预判测试，暂不放入前段普通池</t>
+          <t>教玩家处理易伤与预告爆发，提前防御或爆发击杀</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>旧配置保留；待重命名/重做素材</t>
+          <t>已接入；待生成素材</t>
         </is>
       </c>
     </row>

</xml_diff>